<commit_message>
fix: use degree signals directly for steering/yaw KPIs and simplifiy conversions
</commit_message>
<xml_diff>
--- a/src/config/signal_map.xlsx
+++ b/src/config/signal_map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{174D887F-BED4-0540-966A-2A85889C0BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19569164-10F2-D84D-B4CE-4C3E44AAC1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -882,9 +882,6 @@
       <c r="D6" t="s">
         <v>7</v>
       </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">

</xml_diff>

<commit_message>
add obstacle decoding and multi-row cycle dashboard with speed-colored path
</commit_message>
<xml_diff>
--- a/src/config/signal_map.xlsx
+++ b/src/config/signal_map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19569164-10F2-D84D-B4CE-4C3E44AAC1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2235FF20-97B6-0B49-9FE8-05E06FE126BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="139">
   <si>
     <t>raster</t>
   </si>
@@ -125,9 +125,6 @@
     <t>aeb_state_info/most_relevant_object_id</t>
   </si>
   <si>
-    <t>targetId</t>
-  </si>
-  <si>
     <t>aeb_state_info/time_to_collision</t>
   </si>
   <si>
@@ -405,6 +402,42 @@
   </si>
   <si>
     <t>rad/s</t>
+  </si>
+  <si>
+    <t>objectFused</t>
+  </si>
+  <si>
+    <t>obstacle/confidence</t>
+  </si>
+  <si>
+    <t>obstConf</t>
+  </si>
+  <si>
+    <t>obstacle/position_confidence/confidence</t>
+  </si>
+  <si>
+    <t>posConf</t>
+  </si>
+  <si>
+    <t>obstacle/velocity_confidence/confidence</t>
+  </si>
+  <si>
+    <t>velConf</t>
+  </si>
+  <si>
+    <t>aebTargetId</t>
+  </si>
+  <si>
+    <t>fcwTargetId</t>
+  </si>
+  <si>
+    <t>fcw_state_info/most_relevant_object_id</t>
+  </si>
+  <si>
+    <t>target_obstacle_class</t>
+  </si>
+  <si>
+    <t>aebTargetType</t>
   </si>
 </sst>
 </file>
@@ -781,7 +814,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.1640625" bestFit="1" customWidth="1"/>
@@ -804,7 +837,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -849,7 +882,7 @@
         <v>7</v>
       </c>
       <c r="E4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -866,7 +899,7 @@
         <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -925,7 +958,7 @@
         <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -942,7 +975,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -959,7 +992,7 @@
         <v>7</v>
       </c>
       <c r="E11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -984,10 +1017,10 @@
         <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>134</v>
       </c>
       <c r="D13" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -995,13 +1028,13 @@
         <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
+        <v>136</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>135</v>
       </c>
       <c r="D14" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -1009,13 +1042,13 @@
         <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D15" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -1023,94 +1056,94 @@
         <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C18" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" t="s">
         <v>44</v>
       </c>
-      <c r="B19" t="s">
-        <v>47</v>
-      </c>
       <c r="C19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B21" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D21" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D22" t="s">
         <v>7</v>
@@ -1118,41 +1151,41 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D23" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D24" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" t="s">
         <v>57</v>
       </c>
-      <c r="B25" t="s">
-        <v>60</v>
-      </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D25" t="s">
         <v>7</v>
@@ -1160,153 +1193,153 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="C26" t="s">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="D26" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B27" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C27" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B28" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D28" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B29" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C29" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B30" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C30" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B31" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C31" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B32" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C32" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D32" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B33" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C33" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D33" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B34" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C34" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D34" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>108</v>
+        <v>49</v>
       </c>
       <c r="B35" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C35" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D35" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>107</v>
+      </c>
+      <c r="B36" t="s">
         <v>108</v>
       </c>
-      <c r="B36" t="s">
-        <v>110</v>
-      </c>
       <c r="C36" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D36" t="s">
         <v>7</v>
@@ -1314,16 +1347,16 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>30</v>
+        <v>107</v>
       </c>
       <c r="B37" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C37" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D37" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -1331,75 +1364,145 @@
         <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C38" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D38" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="B39" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C39" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D39" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C40" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D40" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B41" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C41" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B42" t="s">
+        <v>118</v>
+      </c>
+      <c r="C42" t="s">
+        <v>119</v>
+      </c>
+      <c r="D42" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B43" t="s">
+        <v>120</v>
+      </c>
+      <c r="C43" t="s">
         <v>121</v>
       </c>
-      <c r="C42" t="s">
-        <v>122</v>
-      </c>
-      <c r="D42" t="s">
-        <v>39</v>
+      <c r="D43" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>127</v>
+      </c>
+      <c r="B44" t="s">
+        <v>128</v>
+      </c>
+      <c r="C44" t="s">
+        <v>129</v>
+      </c>
+      <c r="D44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>127</v>
+      </c>
+      <c r="B45" t="s">
+        <v>130</v>
+      </c>
+      <c r="C45" t="s">
+        <v>131</v>
+      </c>
+      <c r="D45" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>127</v>
+      </c>
+      <c r="B46" t="s">
+        <v>132</v>
+      </c>
+      <c r="C46" t="s">
+        <v>133</v>
+      </c>
+      <c r="D46" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>30</v>
+      </c>
+      <c r="B47" t="s">
+        <v>137</v>
+      </c>
+      <c r="C47" t="s">
+        <v>138</v>
+      </c>
+      <c r="D47" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1 A26:D36 A7:D8 A6:B6 D6 A12:D25 A9:B9 D9 A10:B10 D10 A11:B11 D11 A3:D5 A2:B2 D2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D1 A7:D8 A6:B6 D6 A15:D37 A9:B11 D9:D11 A3:D5 A2:B2 D2 A12:D12 A13:B13" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1518,38 +1621,38 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" t="s">
         <v>42</v>
       </c>
-      <c r="C8" t="s">
-        <v>43</v>
-      </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" t="s">
         <v>62</v>
       </c>
-      <c r="C9" t="s">
-        <v>63</v>
-      </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" t="s">
         <v>64</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>65</v>
-      </c>
-      <c r="C10" t="s">
-        <v>66</v>
       </c>
       <c r="D10" t="s">
         <v>7</v>
@@ -1557,13 +1660,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
         <v>67</v>
-      </c>
-      <c r="C11" t="s">
-        <v>68</v>
       </c>
       <c r="D11" t="s">
         <v>7</v>
@@ -1574,10 +1677,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" t="s">
         <v>69</v>
-      </c>
-      <c r="C12" t="s">
-        <v>70</v>
       </c>
       <c r="D12" t="s">
         <v>7</v>
@@ -1585,16 +1688,16 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" t="s">
         <v>71</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>72</v>
-      </c>
-      <c r="D13" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -1602,108 +1705,108 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" t="s">
         <v>74</v>
       </c>
-      <c r="C14" t="s">
-        <v>75</v>
-      </c>
       <c r="D14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" t="s">
         <v>76</v>
       </c>
-      <c r="C15" t="s">
-        <v>77</v>
-      </c>
       <c r="D15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" t="s">
         <v>78</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>79</v>
       </c>
-      <c r="C16" t="s">
-        <v>80</v>
-      </c>
       <c r="D16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" t="s">
         <v>81</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>82</v>
-      </c>
-      <c r="D17" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" t="s">
         <v>84</v>
       </c>
-      <c r="C18" t="s">
-        <v>85</v>
-      </c>
       <c r="D18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B19" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19" t="s">
         <v>86</v>
       </c>
-      <c r="C19" t="s">
-        <v>87</v>
-      </c>
       <c r="D19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" t="s">
         <v>88</v>
       </c>
-      <c r="C20" t="s">
-        <v>89</v>
-      </c>
       <c r="D20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>107</v>
+      </c>
+      <c r="B21" t="s">
         <v>108</v>
       </c>
-      <c r="B21" t="s">
-        <v>109</v>
-      </c>
       <c r="C21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D21" t="s">
         <v>7</v>
@@ -1711,13 +1814,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D22" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
add AEB-FB path to visualize feature state
</commit_message>
<xml_diff>
--- a/src/config/signal_map.xlsx
+++ b/src/config/signal_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB29D72E-DB07-C348-AA01-FD6B7CAE8562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0737F8-32F3-CE48-A0A0-59FDE9905EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34420" yWindow="2900" windowWidth="34200" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignalsLong" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="141">
   <si>
     <t>raster</t>
   </si>
@@ -438,6 +438,12 @@
   </si>
   <si>
     <t>aebTargetType</t>
+  </si>
+  <si>
+    <t>fcw_state_info/state</t>
+  </si>
+  <si>
+    <t>fcwState</t>
   </si>
 </sst>
 </file>
@@ -814,7 +820,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.1640625" bestFit="1" customWidth="1"/>
@@ -1081,13 +1087,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>41</v>
+        <v>139</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>140</v>
       </c>
       <c r="D18" t="s">
         <v>38</v>
@@ -1095,13 +1101,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D19" t="s">
         <v>38</v>
@@ -1112,10 +1118,10 @@
         <v>43</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C20" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D20" t="s">
         <v>38</v>
@@ -1126,10 +1132,10 @@
         <v>43</v>
       </c>
       <c r="B21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D21" t="s">
         <v>38</v>
@@ -1137,27 +1143,27 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C22" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D22" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D23" t="s">
         <v>7</v>
@@ -1165,30 +1171,30 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D24" t="s">
-        <v>38</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C25" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D25" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -1196,10 +1202,10 @@
         <v>56</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C26" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D26" t="s">
         <v>7</v>
@@ -1207,16 +1213,16 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B27" t="s">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D27" t="s">
-        <v>82</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -1224,10 +1230,10 @@
         <v>49</v>
       </c>
       <c r="B28" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C28" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D28" t="s">
         <v>82</v>
@@ -1238,10 +1244,10 @@
         <v>49</v>
       </c>
       <c r="B29" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D29" t="s">
         <v>82</v>
@@ -1252,10 +1258,10 @@
         <v>49</v>
       </c>
       <c r="B30" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C30" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D30" t="s">
         <v>82</v>
@@ -1266,10 +1272,10 @@
         <v>49</v>
       </c>
       <c r="B31" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C31" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D31" t="s">
         <v>82</v>
@@ -1280,10 +1286,10 @@
         <v>49</v>
       </c>
       <c r="B32" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C32" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D32" t="s">
         <v>82</v>
@@ -1294,10 +1300,10 @@
         <v>49</v>
       </c>
       <c r="B33" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C33" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D33" t="s">
         <v>82</v>
@@ -1308,10 +1314,10 @@
         <v>49</v>
       </c>
       <c r="B34" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C34" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D34" t="s">
         <v>82</v>
@@ -1322,10 +1328,10 @@
         <v>49</v>
       </c>
       <c r="B35" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C35" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D35" t="s">
         <v>82</v>
@@ -1333,16 +1339,16 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>107</v>
+        <v>49</v>
       </c>
       <c r="B36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C36" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D36" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
@@ -1350,10 +1356,10 @@
         <v>107</v>
       </c>
       <c r="B37" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C37" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D37" t="s">
         <v>7</v>
@@ -1361,16 +1367,16 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>30</v>
+        <v>107</v>
       </c>
       <c r="B38" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C38" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D38" t="s">
-        <v>82</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
@@ -1378,10 +1384,10 @@
         <v>30</v>
       </c>
       <c r="B39" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C39" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D39" t="s">
         <v>82</v>
@@ -1389,16 +1395,16 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B40" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C40" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D40" t="s">
-        <v>38</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
@@ -1406,10 +1412,10 @@
         <v>49</v>
       </c>
       <c r="B41" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C41" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D41" t="s">
         <v>38</v>
@@ -1420,10 +1426,10 @@
         <v>49</v>
       </c>
       <c r="B42" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C42" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D42" t="s">
         <v>38</v>
@@ -1434,10 +1440,10 @@
         <v>49</v>
       </c>
       <c r="B43" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C43" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D43" t="s">
         <v>38</v>
@@ -1445,16 +1451,16 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>127</v>
+        <v>49</v>
       </c>
       <c r="B44" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C44" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D44" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
@@ -1462,10 +1468,10 @@
         <v>127</v>
       </c>
       <c r="B45" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C45" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D45" t="s">
         <v>7</v>
@@ -1476,10 +1482,10 @@
         <v>127</v>
       </c>
       <c r="B46" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C46" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D46" t="s">
         <v>7</v>
@@ -1487,22 +1493,36 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
+        <v>127</v>
+      </c>
+      <c r="B47" t="s">
+        <v>132</v>
+      </c>
+      <c r="C47" t="s">
+        <v>133</v>
+      </c>
+      <c r="D47" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
         <v>30</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B48" t="s">
         <v>137</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C48" t="s">
         <v>138</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D48" t="s">
         <v>82</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1 A7:D8 A6:B6 D6 A15:D37 A9:B11 D9:D11 A3:D5 A2:B2 D2 A12:B12 A13:B13 D12" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D1 A7:D8 A6:B6 D6 A19:D38 A3:D5 A2:B2 D2 A9:B13 D9:D12 A15:D17" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
aeb val and rov availability check added
</commit_message>
<xml_diff>
--- a/src/config/signal_map.xlsx
+++ b/src/config/signal_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0737F8-32F3-CE48-A0A0-59FDE9905EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DC27D26-18C1-3943-BAA5-EE8DF3E23460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34420" yWindow="2900" windowWidth="34200" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34200" yWindow="600" windowWidth="38400" windowHeight="23400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignalsLong" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="145">
   <si>
     <t>raster</t>
   </si>
@@ -444,6 +444,18 @@
   </si>
   <si>
     <t>fcwState</t>
+  </si>
+  <si>
+    <t>aeb_state_info/degradation</t>
+  </si>
+  <si>
+    <t>aebDegradation</t>
+  </si>
+  <si>
+    <t>active_safety_settings/AEB/configuration_level</t>
+  </si>
+  <si>
+    <t>aebConfigLvl</t>
   </si>
 </sst>
 </file>
@@ -820,7 +832,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.1640625" bestFit="1" customWidth="1"/>
@@ -1171,13 +1183,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
-        <v>52</v>
+        <v>143</v>
       </c>
       <c r="C24" t="s">
-        <v>53</v>
+        <v>144</v>
       </c>
       <c r="D24" t="s">
         <v>7</v>
@@ -1185,30 +1197,30 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C25" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D25" t="s">
-        <v>38</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C26" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D26" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -1216,10 +1228,10 @@
         <v>56</v>
       </c>
       <c r="B27" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D27" t="s">
         <v>7</v>
@@ -1227,16 +1239,16 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B28" t="s">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D28" t="s">
-        <v>82</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -1244,10 +1256,10 @@
         <v>49</v>
       </c>
       <c r="B29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C29" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D29" t="s">
         <v>82</v>
@@ -1258,10 +1270,10 @@
         <v>49</v>
       </c>
       <c r="B30" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C30" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D30" t="s">
         <v>82</v>
@@ -1272,10 +1284,10 @@
         <v>49</v>
       </c>
       <c r="B31" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C31" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D31" t="s">
         <v>82</v>
@@ -1286,10 +1298,10 @@
         <v>49</v>
       </c>
       <c r="B32" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C32" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D32" t="s">
         <v>82</v>
@@ -1300,10 +1312,10 @@
         <v>49</v>
       </c>
       <c r="B33" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C33" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D33" t="s">
         <v>82</v>
@@ -1314,10 +1326,10 @@
         <v>49</v>
       </c>
       <c r="B34" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C34" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D34" t="s">
         <v>82</v>
@@ -1328,10 +1340,10 @@
         <v>49</v>
       </c>
       <c r="B35" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C35" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D35" t="s">
         <v>82</v>
@@ -1342,10 +1354,10 @@
         <v>49</v>
       </c>
       <c r="B36" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C36" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D36" t="s">
         <v>82</v>
@@ -1353,16 +1365,16 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>107</v>
+        <v>49</v>
       </c>
       <c r="B37" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C37" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D37" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -1370,10 +1382,10 @@
         <v>107</v>
       </c>
       <c r="B38" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C38" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D38" t="s">
         <v>7</v>
@@ -1381,16 +1393,16 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>30</v>
+        <v>107</v>
       </c>
       <c r="B39" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C39" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D39" t="s">
-        <v>82</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
@@ -1398,10 +1410,10 @@
         <v>30</v>
       </c>
       <c r="B40" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C40" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D40" t="s">
         <v>82</v>
@@ -1409,16 +1421,16 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B41" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C41" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D41" t="s">
-        <v>38</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
@@ -1426,10 +1438,10 @@
         <v>49</v>
       </c>
       <c r="B42" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C42" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D42" t="s">
         <v>38</v>
@@ -1440,10 +1452,10 @@
         <v>49</v>
       </c>
       <c r="B43" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C43" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D43" t="s">
         <v>38</v>
@@ -1454,10 +1466,10 @@
         <v>49</v>
       </c>
       <c r="B44" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C44" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D44" t="s">
         <v>38</v>
@@ -1465,16 +1477,16 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>127</v>
+        <v>49</v>
       </c>
       <c r="B45" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C45" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D45" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
@@ -1482,10 +1494,10 @@
         <v>127</v>
       </c>
       <c r="B46" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C46" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D46" t="s">
         <v>7</v>
@@ -1496,10 +1508,10 @@
         <v>127</v>
       </c>
       <c r="B47" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C47" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D47" t="s">
         <v>7</v>
@@ -1507,22 +1519,50 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
+        <v>127</v>
+      </c>
+      <c r="B48" t="s">
+        <v>132</v>
+      </c>
+      <c r="C48" t="s">
+        <v>133</v>
+      </c>
+      <c r="D48" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>30</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B49" t="s">
         <v>137</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C49" t="s">
         <v>138</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D49" t="s">
         <v>82</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>30</v>
+      </c>
+      <c r="B50" t="s">
+        <v>141</v>
+      </c>
+      <c r="C50" t="s">
+        <v>142</v>
+      </c>
+      <c r="D50" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1 A7:D8 A6:B6 D6 A19:D38 A3:D5 A2:B2 D2 A9:B13 D9:D12 A15:D17" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D1 A7:D8 A6:B6 D6 A25:D39 A3:D5 A2:B2 D2 A9:B13 D9:D12 A15:D17 A19:D23" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
cycle KPI top_figure optimized
</commit_message>
<xml_diff>
--- a/src/config/signal_map.xlsx
+++ b/src/config/signal_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DC27D26-18C1-3943-BAA5-EE8DF3E23460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76851A2E-02ED-804C-8B68-F1E832012950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34200" yWindow="600" windowWidth="38400" windowHeight="23400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="53680" yWindow="3220" windowWidth="22160" windowHeight="23400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignalsLong" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Refactor cycle KPI extractors
</commit_message>
<xml_diff>
--- a/src/config/signal_map.xlsx
+++ b/src/config/signal_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76851A2E-02ED-804C-8B68-F1E832012950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A73BD7-9F97-574B-BFA7-B3BA99977108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="53680" yWindow="3220" windowWidth="22160" windowHeight="23400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37380" yWindow="8540" windowWidth="37380" windowHeight="23400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignalsLong" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
clarify KPI rules in extractors; update requirements and PyInstaller spec
</commit_message>
<xml_diff>
--- a/src/config/signal_map.xlsx
+++ b/src/config/signal_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A73BD7-9F97-574B-BFA7-B3BA99977108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A424E15C-CB95-E04B-BF5D-32B894439FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37380" yWindow="8540" windowWidth="37380" windowHeight="23400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37760" yWindow="2880" windowWidth="29640" windowHeight="20020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignalsLong" sheetId="1" r:id="rId1"/>
@@ -1562,7 +1562,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1 A7:D8 A6:B6 D6 A25:D39 A3:D5 A2:B2 D2 A9:B13 D9:D12 A15:D17 A19:D23" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D1 A7:D8 A6:B6 D6 A25:D30 A3:D5 A2:B2 D2 A9:B13 D9:D12 A15:D17 A19:D23 A32:D39 A31:B31 D31" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>